<commit_message>
Registrar análisis comercial y financiero de las 3 propuestas (128-2026)
Incorpora la Política de Compras (POL-ABA-01) como insumo. Calcula el
criterio Precio con la fórmula y peso oficial de la matriz (40%),
documenta condiciones de pago/plazos/garantías/SLA como observaciones
y alertas, y confirma la inadmisibilidad de precio del Oferente C. La
Minuta Confidencial de Negociación se mantiene excluida de la
calificación, conforme al punto 7 de la Política de Compras.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F1ibwH83Z2BnBsdQki73QB
</commit_message>
<xml_diff>
--- a/agente-procurement/outputs/scorecard_tecnico_128-2026.xlsx
+++ b/agente-procurement/outputs/scorecard_tecnico_128-2026.xlsx
@@ -997,11 +997,17 @@
           <t>Precio Ofertado (CLP) — ingresar valor de la propuesta</t>
         </is>
       </c>
-      <c r="E7" s="53" t="n"/>
+      <c r="E7" s="53" t="n">
+        <v>179800000</v>
+      </c>
       <c r="F7" s="54" t="n"/>
-      <c r="G7" s="53" t="n"/>
+      <c r="G7" s="53" t="n">
+        <v>188900000</v>
+      </c>
       <c r="H7" s="54" t="n"/>
-      <c r="I7" s="53" t="n"/>
+      <c r="I7" s="53" t="n">
+        <v>197200000</v>
+      </c>
       <c r="J7" s="54" t="n"/>
     </row>
     <row r="8" ht="30" customHeight="1" s="38">
@@ -1620,9 +1626,9 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>NOTA: Precio Ofertado (fila 7-8) queda pendiente para la etapa de análisis comercial (03_analisis_comercial.md). Este scorecard cubre exclusivamente los criterios técnicos de la matriz (Experiencia 25%, Plazo 15%, Cumplimiento técnico 20% = 60% del total).</t>
+      <c r="A32" s="37" t="inlineStr">
+        <is>
+          <t>ACTUALIZACIÓN — Análisis comercial: fila 7-8 (Precio) completada con los valores ofertados. Oferente C (columna I) es NO ADMISIBLE por precio (excede en 5,74% el presupuesto referencial, sobre el margen máximo de 5% del punto 3 de las Bases / punto 5 de la Política de Compras POL-ABA-01). Se mantiene su nota calculada solo para trazabilidad.</t>
         </is>
       </c>
     </row>

</xml_diff>